<commit_message>
update from Karina's house
</commit_message>
<xml_diff>
--- a/New tracking file.xlsx
+++ b/New tracking file.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alonso\Documents\GitHub\Trading\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zuriel\Documents\github\Trading\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F7105FA-96F3-4165-BD4D-16AE6BEDB094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E618D1C-DA77-4D41-9B56-C02ADC3ED6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{045517DB-0C92-4CAE-B507-36AB229E2600}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{045517DB-0C92-4CAE-B507-36AB229E2600}"/>
   </bookViews>
   <sheets>
     <sheet name="Trades" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="112">
   <si>
     <t>Trade_ID</t>
   </si>
@@ -374,6 +374,12 @@
   </si>
   <si>
     <t>T-014</t>
+  </si>
+  <si>
+    <t>T-009</t>
+  </si>
+  <si>
+    <t>T-007</t>
   </si>
 </sst>
 </file>
@@ -1132,11 +1138,11 @@
         <v>55.919999999999959</v>
       </c>
       <c r="L8" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="M8">
         <f>SUMIF(Executions!B:B,A8,Executions!H:H)</f>
-        <v>0</v>
+        <v>-28.16999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -1222,11 +1228,11 @@
         <v>43.539999999999992</v>
       </c>
       <c r="L10" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="M10">
         <f>SUMIF(Executions!B:B,A10,Executions!H:H)</f>
-        <v>0</v>
+        <v>-25.445000000000011</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1492,7 +1498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD56475-86FC-4B41-8DB1-3EDC95E09B14}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
@@ -1564,7 +1570,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <f t="shared" ref="A3:A9" si="0">ROW()-1</f>
+        <f t="shared" ref="A3:A11" si="0">ROW()-1</f>
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -1771,8 +1777,9 @@
       <c r="C9" s="1">
         <v>46087</v>
       </c>
-      <c r="D9" t="s">
-        <v>108</v>
+      <c r="D9" t="str">
+        <f>VLOOKUP(B9,Trades!A$1:M100007,3,FALSE)</f>
+        <v>LULU</v>
       </c>
       <c r="E9" t="s">
         <v>64</v>
@@ -1792,12 +1799,78 @@
         <v>-0.71825396825396837</v>
       </c>
     </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="1">
+        <v>46087</v>
+      </c>
+      <c r="D10" t="str">
+        <f>VLOOKUP(B10,Trades!A$1:M100008,3,FALSE)</f>
+        <v>UUUU</v>
+      </c>
+      <c r="E10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10">
+        <v>18.824999999999999</v>
+      </c>
+      <c r="G10">
+        <v>7</v>
+      </c>
+      <c r="H10">
+        <f>IF(VLOOKUP(B10,Trades!A:M,4,FALSE)="Long",(F10-VLOOKUP(B10,Trades!A:M,6,FALSE))*G10,(VLOOKUP(B10,Trades!A:M,6,FALSE)-F10)*G10)</f>
+        <v>-25.445000000000011</v>
+      </c>
+      <c r="I10">
+        <f>H10/Trades!I10</f>
+        <v>-1.1688102893890682</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="1">
+        <v>46087</v>
+      </c>
+      <c r="D11" t="str">
+        <f>VLOOKUP(B11,Trades!A$1:M100009,3,FALSE)</f>
+        <v>OKLO</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11">
+        <v>58.43</v>
+      </c>
+      <c r="G11">
+        <v>3</v>
+      </c>
+      <c r="H11">
+        <f>IF(VLOOKUP(B11,Trades!A:M,4,FALSE)="Long",(F11-VLOOKUP(B11,Trades!A:M,6,FALSE))*G11,(VLOOKUP(B11,Trades!A:M,6,FALSE)-F11)*G11)</f>
+        <v>-28.16999999999998</v>
+      </c>
+      <c r="I11">
+        <f>H11/Trades!I11</f>
+        <v>-1.2570281124497982</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E1048576" xr:uid="{05958E25-911C-4ED3-A0F6-7B25054B7856}">
-      <formula1>$E$2:$E100009</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E12:E1048576" xr:uid="{05958E25-911C-4ED3-A0F6-7B25054B7856}">
+      <formula1>$E$2:$E100011</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E9" xr:uid="{9C25687B-DEF5-4411-BA9A-40CB4D950704}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E11" xr:uid="{9C25687B-DEF5-4411-BA9A-40CB4D950704}">
       <formula1>"Sell,Cover"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2121,7 +2194,7 @@
       </c>
       <c r="D9">
         <f>COUNTIFS(Trades!E:E, A9, Trades!M:M, "&lt;0")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <f>IFERROR(C9/B9,0)</f>
@@ -2129,19 +2202,19 @@
       </c>
       <c r="F9">
         <f>SUMIF(Trades!E:E,A9,Trades!M:M)</f>
-        <v>87.110000000000056</v>
+        <v>61.665000000000049</v>
       </c>
       <c r="G9">
         <f t="shared" si="1"/>
-        <v>17.422000000000011</v>
+        <v>12.333000000000009</v>
       </c>
       <c r="H9">
         <f>IFERROR( SUMIFS(Trades!M:M, Trades!E:E, A9, Trades!M:M, "&gt;0")/ABS(SUMIFS(Trades!M:M, Trades!E:E, A9, Trades!M:M,"&lt;0")),0)</f>
-        <v>0</v>
+        <v>3.4234623698172535</v>
       </c>
       <c r="I9">
         <f t="shared" si="2"/>
-        <v>17.422000000000011</v>
+        <v>12.333000000000009</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -2158,7 +2231,7 @@
       </c>
       <c r="D10">
         <f>COUNTIFS(Trades!E:E, A10, Trades!M:M, "&lt;0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10">
         <f>IFERROR(C10/B10,0)</f>
@@ -2166,11 +2239,11 @@
       </c>
       <c r="F10">
         <f>SUMIF(Trades!E:E,A10,Trades!M:M)</f>
-        <v>-55.721999999999952</v>
+        <v>-83.891999999999939</v>
       </c>
       <c r="G10">
         <f>IFERROR(F10/B10,0)</f>
-        <v>-11.14439999999999</v>
+        <v>-16.778399999999987</v>
       </c>
       <c r="H10">
         <f>IFERROR( SUMIFS(Trades!M:M, Trades!E:E, A10, Trades!M:M, "&gt;0")/ABS(SUMIFS(Trades!M:M, Trades!E:E, A10, Trades!M:M,"&lt;0")),0)</f>
@@ -2178,7 +2251,7 @@
       </c>
       <c r="I10">
         <f>IFERROR(F10/B10,0)</f>
-        <v>-11.14439999999999</v>
+        <v>-16.778399999999987</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2526,7 +2599,7 @@
       </c>
       <c r="B4">
         <f>AVERAGE(Trades!M:M)</f>
-        <v>8.2227142857143054</v>
+        <v>4.3930714285714485</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2535,7 +2608,7 @@
       </c>
       <c r="B5">
         <f>SUM(Trades!M:M)</f>
-        <v>115.11800000000028</v>
+        <v>61.503000000000284</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2544,7 +2617,7 @@
       </c>
       <c r="B6">
         <f>SUMIF(Trades!M:M,"&gt;0")/ABS(SUM(Trades!M:M,""&lt;0))</f>
-        <v>1.4840424607793723</v>
+        <v>2.7777506788286654</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2567,7 +2640,7 @@
       </c>
       <c r="B10">
         <f>MIN(Trades!M:M)</f>
-        <v>-23.399999999999981</v>
+        <v>-28.16999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2585,7 +2658,7 @@
       </c>
       <c r="B12">
         <f>AVERAGEIF(Trades!M:M,"&lt;0")</f>
-        <v>-18.573999999999984</v>
+        <v>-21.867399999999989</v>
       </c>
     </row>
   </sheetData>

</xml_diff>